<commit_message>
DATA_TESTS (two tests, done)
</commit_message>
<xml_diff>
--- a/Data/0_task_01_claims.xlsx
+++ b/Data/0_task_01_claims.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\minam\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\Lux_Project_Intern\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{4FBB2839-C4C8-4060-A3CB-A232691408BB}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="10_ncr:8100000_{3E29646C-09AE-4083-9D1A-3E1A97F02490}" xr6:coauthVersionLast="32" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8952" activeTab="3" xr2:uid="{65A2B071-1A6E-46E7-B634-5A08B92D1495}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8952" xr2:uid="{65A2B071-1A6E-46E7-B634-5A08B92D1495}"/>
   </bookViews>
   <sheets>
     <sheet name="Data" sheetId="1" r:id="rId1"/>
@@ -943,19 +943,19 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="167" formatCode="dd/mm/yyyy"/>
+      <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="19" formatCode="m/d/yyyy"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -974,15 +974,15 @@
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{BD85A2A9-CBCF-401E-B362-1405FBB3BDF9}" name="Table1" displayName="Table1" ref="A1:I84" totalsRowShown="0">
   <autoFilter ref="A1:I84" xr:uid="{BD85A2A9-CBCF-401E-B362-1405FBB3BDF9}"/>
   <tableColumns count="9">
-    <tableColumn id="1" xr3:uid="{5CC5547C-430E-4A69-B3E8-5472F3753CF4}" name="As of" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{5CC5547C-430E-4A69-B3E8-5472F3753CF4}" name="As of" dataDxfId="4"/>
     <tableColumn id="2" xr3:uid="{43023757-C05B-4959-A1E6-5BF0BD91C13E}" name="POL_No"/>
     <tableColumn id="3" xr3:uid="{4AABDED0-A340-40E1-B5E6-840BFFEC8B8A}" name="Claim_No"/>
     <tableColumn id="6" xr3:uid="{237815BA-4632-4052-B592-8E7EF6404374}" name="Major Line of Buisness"/>
-    <tableColumn id="8" xr3:uid="{10818BA2-7E82-4F51-91E6-F6C0F34D685A}" name="Accindent Date" dataDxfId="4"/>
-    <tableColumn id="10" xr3:uid="{B8DD90A5-56A1-4B2D-A5C6-418C7CA0A56F}" name="Paid Date" dataDxfId="3"/>
+    <tableColumn id="8" xr3:uid="{10818BA2-7E82-4F51-91E6-F6C0F34D685A}" name="Accindent Date" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{B8DD90A5-56A1-4B2D-A5C6-418C7CA0A56F}" name="Paid Date" dataDxfId="2"/>
     <tableColumn id="12" xr3:uid="{2EE81387-F82F-4D53-925B-21FF0B6CC01B}" name="status"/>
-    <tableColumn id="13" xr3:uid="{47C7DFAA-2B9F-497F-8EF1-16BC9DEEA79A}" name="Gross" dataDxfId="2" dataCellStyle="Comma"/>
-    <tableColumn id="14" xr3:uid="{D042D151-7B0E-4C3A-8DB5-0F2C311CFB1B}" name="Ceded" dataDxfId="1" dataCellStyle="Comma"/>
+    <tableColumn id="13" xr3:uid="{47C7DFAA-2B9F-497F-8EF1-16BC9DEEA79A}" name="Gross" dataDxfId="1" dataCellStyle="Comma"/>
+    <tableColumn id="14" xr3:uid="{D042D151-7B0E-4C3A-8DB5-0F2C311CFB1B}" name="Ceded" dataDxfId="0" dataCellStyle="Comma"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight9" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3903,7 +3903,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAF9C9AE-5995-4621-8A1F-5899CA7EAF6E}">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="20.296875" bestFit="1" customWidth="1"/>
@@ -4023,8 +4023,6 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:5"/>
-    <row r="7" spans="1:5"/>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>